<commit_message>
task-2360: fit to pages estimate, manual breaks with fit, row heights by the point, unreadable break lists by count
</commit_message>
<xml_diff>
--- a/crates/unluminous-sheet/tests/fixtures/pages/pages-aptos-narrow.xlsx
+++ b/crates/unluminous-sheet/tests/fixtures/pages/pages-aptos-narrow.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\jason\dev\unluminous\.claude\worktrees\agent-afa636fef9f2b0676\crates\unluminous-sheet\tests\fixtures\pages\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{27A631F4-2982-429F-B2ED-85AB0610F9E7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{196855A8-6B5F-484B-98E4-82B96E5A8E20}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1875" yWindow="6660" windowWidth="43200" windowHeight="23445" activeTab="6" xr2:uid="{98C7AFF7-03EE-4041-9E81-C8503A5BC1B4}"/>
+    <workbookView xWindow="1875" yWindow="6660" windowWidth="43200" windowHeight="23445" activeTab="6" xr2:uid="{FB48A966-886D-49F8-BC2C-7ED0737EC33F}"/>
   </bookViews>
   <sheets>
     <sheet name="letter-p" sheetId="1" r:id="rId1"/>
@@ -413,7 +413,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F2FB63B8-60FD-440E-8585-22B1401E45D2}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6F37E3E9-7520-4D54-AD61-2F479419D4BE}">
   <dimension ref="A1:AN130"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -16284,7 +16284,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{79911C86-574C-494D-8AFC-C94409BE11A4}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DC682BB6-79AF-43CD-93F9-7A04C7866296}">
   <dimension ref="A1:AN130"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -32155,7 +32155,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B738D745-88E1-49D5-9F92-373D50A01243}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8DC83329-55AB-4002-8162-500709219A65}">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
@@ -48029,7 +48029,7 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C6988BD0-FF93-430E-95FF-2F6C59BF244F}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C1F5CC1F-BAD1-4A88-BBCC-95865BB4D33F}">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
@@ -63903,7 +63903,7 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2FDA17F6-A299-4080-8EEF-8A135AA8A9BF}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D5C63389-FC34-4314-8593-173C9C93B185}">
   <dimension ref="A1:AN130"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -79774,7 +79774,7 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7B84D63B-EA62-4210-B803-5B373B2ADE77}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E7C5A81A-E7F0-4C00-8435-AFC45B861E20}">
   <dimension ref="A1:AN130"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -95645,7 +95645,7 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{33A0303F-71FD-4A1D-9DD3-BA9B58B12179}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BD9A0B86-1A45-432A-8F6E-94B2403B35FA}">
   <dimension ref="A1:AN130"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>

</xml_diff>